<commit_message>
Add header block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 14
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,6 +37,27 @@
     <t>url</t>
   </si>
   <si>
+    <t>coming-soon.report.json</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>coming-soon</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>2026-09-28T10:24:07.088Z</t>
+  </si>
+  <si>
+    <t>Coming soon | Kapoor Jewellers</t>
+  </si>
+  <si>
+    <t>https://www.tanishq.com/homepage</t>
+  </si>
+  <si>
     <t>homepage.report.json</t>
   </si>
   <si>
@@ -46,16 +67,19 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
-    <t>2026-09-28T10:14:31.795Z</t>
+    <t>2026-09-28T10:17:16.485Z</t>
   </si>
   <si>
     <t>Buy Latest Gold and Diamond Jewelry Online by Kapoor Jewellers USA</t>
   </si>
   <si>
-    <t>https://www.tanishq.com/homepage</t>
+    <t>index.report.json</t>
+  </si>
+  <si>
+    <t>index</t>
+  </si>
+  <si>
+    <t>2026-09-28T10:24:43.797Z</t>
   </si>
 </sst>
 </file>
@@ -444,13 +468,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="50" customWidth="1"/>
     <col min="8" max="8" width="34" customWidth="1"/>
@@ -508,6 +532,58 @@
         <v>14</v>
       </c>
     </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add footer, header blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 11
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -49,7 +49,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-09-28T10:24:07.088Z</t>
+    <t>2026-09-28T10:29:26.049Z</t>
   </si>
   <si>
     <t>Coming soon | Kapoor Jewellers</t>
@@ -79,7 +79,7 @@
     <t>index</t>
   </si>
   <si>
-    <t>2026-09-28T10:24:43.797Z</t>
+    <t>2026-09-28T11:41:05.851Z</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
POC shop and Experience Platform tracking for Earrings and Rings
- Shop blocks: product-list, product-details, cart, checkout, account; catalogue in
  data/products.json (built from the homepage products); cart, test accounts and
  test orders kept in the browser
- Tracking per docs/tracking-spec.md: page views, link clicks, commerce and account
  events, consent and profile records; Web SDK loads only after cookie consent and
  stays in dry-run until the datastream ID is configured
- Header bag icon shows the cart count; homepage product cards open the product page
- Preview helpers: internal links follow /content in the local/aemcoder preview,
  404 redirects stay inside it, ?tracking-debug=1 shows an on-page event viewer
- Importer: shop page imports and product-link rewrite

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="53">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,6 +19,12 @@
     <t>blocks</t>
   </si>
   <si>
+    <t>error</t>
+  </si>
+  <si>
+    <t>errorStack</t>
+  </si>
+  <si>
     <t>path</t>
   </si>
   <si>
@@ -37,49 +43,139 @@
     <t>url</t>
   </si>
   <si>
+    <t>account.report.json</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>account</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>shop</t>
+  </si>
+  <si>
+    <t>2026-10-02T11:28:02.765Z</t>
+  </si>
+  <si>
+    <t>My account | Kapoor Jewellers</t>
+  </si>
+  <si>
+    <t>https://www.tanishq.com/homepage</t>
+  </si>
+  <si>
+    <t>cart.report.json</t>
+  </si>
+  <si>
+    <t>cart</t>
+  </si>
+  <si>
+    <t>2026-10-02T11:27:46.664Z</t>
+  </si>
+  <si>
+    <t>Your cart | Kapoor Jewellers</t>
+  </si>
+  <si>
+    <t>checkout.report.json</t>
+  </si>
+  <si>
+    <t>checkout</t>
+  </si>
+  <si>
+    <t>2026-10-02T11:27:54.318Z</t>
+  </si>
+  <si>
+    <t>Checkout | Kapoor Jewellers</t>
+  </si>
+  <si>
     <t>coming-soon.report.json</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>coming-soon</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>2026-09-28T10:29:26.049Z</t>
   </si>
   <si>
     <t>Coming soon | Kapoor Jewellers</t>
   </si>
   <si>
-    <t>https://www.tanishq.com/homepage</t>
-  </si>
-  <si>
     <t>homepage.report.json</t>
   </si>
   <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: Cannot read properties of undefined (reading 'replace')
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: Cannot read properties of undefined (reading 'replace')
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30
+    at processUrl (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:693:31)
+    at async main (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:956:22)</t>
+  </si>
+  <si>
+    <t>homepage</t>
+  </si>
+  <si>
+    <t>failed</t>
+  </si>
+  <si>
+    <t>2026-10-02T11:26:40.493Z</t>
+  </si>
+  <si>
+    <t>index.report.json</t>
+  </si>
+  <si>
     <t>["carousel-hero","cards-category","cards-product","cards-product","cards-product","columns-spotlight","cards-video","cards-occasion","cards-collection","columns-audience","columns-showcase","cards-gifting","cards-store"]</t>
   </si>
   <si>
-    <t>homepage</t>
-  </si>
-  <si>
-    <t>2026-09-28T10:17:16.485Z</t>
+    <t>index</t>
+  </si>
+  <si>
+    <t>2026-10-02T11:29:11.073Z</t>
   </si>
   <si>
     <t>Buy Latest Gold and Diamond Jewelry Online by Kapoor Jewellers USA</t>
   </si>
   <si>
-    <t>index.report.json</t>
-  </si>
-  <si>
-    <t>index</t>
-  </si>
-  <si>
-    <t>2026-09-28T11:41:05.851Z</t>
+    <t>product.report.json</t>
+  </si>
+  <si>
+    <t>product</t>
+  </si>
+  <si>
+    <t>2026-10-02T11:27:38.310Z</t>
+  </si>
+  <si>
+    <t>Product | Kapoor Jewellers</t>
+  </si>
+  <si>
+    <t>jewelry/earrings.report.json</t>
+  </si>
+  <si>
+    <t>jewelry/earrings</t>
+  </si>
+  <si>
+    <t>2026-10-02T11:27:21.739Z</t>
+  </si>
+  <si>
+    <t>Earrings | Kapoor Jewellers</t>
+  </si>
+  <si>
+    <t>jewelry/rings.report.json</t>
+  </si>
+  <si>
+    <t>jewelry/rings</t>
+  </si>
+  <si>
+    <t>2026-10-02T11:27:29.641Z</t>
+  </si>
+  <si>
+    <t>Rings | Kapoor Jewellers</t>
   </si>
 </sst>
 </file>
@@ -468,19 +564,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="34" customWidth="1"/>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="4" width="50" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="9" width="50" customWidth="1"/>
+    <col min="10" max="10" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -505,87 +601,303 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
         <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
         <v>13</v>
       </c>
-      <c r="H2" t="s">
+      <c r="G3" t="s">
         <v>14</v>
       </c>
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J4" t="s">
         <v>17</v>
       </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J5" t="s">
         <v>17</v>
       </c>
-      <c r="F3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" t="s">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" t="s">
+        <v>40</v>
+      </c>
+      <c r="J7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" t="s">
         <v>14</v>
       </c>
+      <c r="H8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I8" t="s">
+        <v>44</v>
+      </c>
+      <c r="J8" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
+        <v>47</v>
+      </c>
+      <c r="I9" t="s">
+        <v>48</v>
+      </c>
+      <c r="J9" t="s">
         <v>17</v>
       </c>
-      <c r="F4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" t="s">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" t="s">
         <v>14</v>
+      </c>
+      <c r="H10" t="s">
+        <v>51</v>
+      </c>
+      <c r="I10" t="s">
+        <v>52</v>
+      </c>
+      <c r="J10" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>